<commit_message>
feat: complete pedagogical lecture visualizer redesign, dynamic scope governance, and learning material resources
</commit_message>
<xml_diff>
--- a/output/pms/Lập_trình_Python/Session 04 - Toán tử Số học, Toán tử So sánh và Toán tử Logic trong Python/Lesson 01 - Toán tử Số học và Toán tử Gán/Câu hỏi Quizz/Quizz_Session04_Lesson01.xlsx
+++ b/output/pms/Lập_trình_Python/Session 04 - Toán tử Số học, Toán tử So sánh và Toán tử Logic trong Python/Lesson 01 - Toán tử Số học và Toán tử Gán/Câu hỏi Quizz/Quizz_Session04_Lesson01.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Quizz Questions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quizz Questions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -483,7 +483,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Khi triển khai Toán tử Số học và Toán tử Gán trong dự án `python`, cú pháp khai báo nào sau đây đúng quy chuẩn và đảm bảo chương trình biên dịch/thực thi không báo lỗi?</t>
+          <t>Trong Python, phép toán nào sau đây dùng để chia lấy phần nguyên (floor division) và phép toán nào chia lấy phần dư (modulus)?</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
@@ -491,31 +491,31 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Khai báo cú pháp chuẩn theo quy ước đặt tên của `python`</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>Toán tử / để chia lấy nguyên và % để chia lấy dư.</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n"/>
       <c r="B3" s="4" t="n"/>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Sử dụng từ khóa thuộc phiên bản đã bị loại bỏ (Deprecated)</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="n"/>
+          <t>Toán tử // để chia lấy nguyên và % để chia lấy dư.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n"/>
       <c r="B4" s="4" t="n"/>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bỏ qua việc khởi tạo giá trị ban đầu cho các tham số bắt buộc</t>
+          <t>Toán tử / để chia lấy nguyên và // để chia lấy dư.</t>
         </is>
       </c>
       <c r="D4" s="3" t="n"/>
@@ -525,7 +525,7 @@
       <c r="B5" s="4" t="n"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Đặt tên biến bằng ký tự đặc biệt không được ngôn ngữ hỗ trợ</t>
+          <t>Toán tử // để chia lấy nguyên và mod để chia lấy dư.</t>
         </is>
       </c>
       <c r="D5" s="3" t="n"/>
@@ -533,7 +533,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Trong cơ chế vận hành của Toán tử Số học và Toán tử Gán, luồng thực thi của hệ thống sẽ xử lý như thế nào khi gặp điều kiện rẽ nhánh trả về `False`?</t>
+          <t>Cho đoạn mã sau: `x = 10; y = 3; z = x // y + x % y`. Giá trị của `z` là bao nhiêu?</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
@@ -541,21 +541,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bỏ qua khối lệnh phụ thuộc và tiếp tục thực thi các câu lệnh kế tiếp</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n"/>
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Dừng toàn bộ hệ thống và thoát chương trình lập tức</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D7" s="3" t="n"/>
@@ -565,17 +561,21 @@
       <c r="B8" s="4" t="n"/>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Lặp lại khối lệnh vô tận cho đến khi bộ nhớ RAM bị tràn</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="n"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n"/>
       <c r="B9" s="4" t="n"/>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Tự động sửa đổi giá trị dữ liệu đầu vào cho phù hợp</t>
+          <t>3.3333333333333335</t>
         </is>
       </c>
       <c r="D9" s="3" t="n"/>
@@ -583,13 +583,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Cho đoạn mã nguồn minh họa Toán tử Số học và Toán tử Gán trong `python`:
-```python
-# Đoạn mã nguồn minh họa luồng xử lý
-result = process_data(input_val=100)
-print(result)
-```python
-Kết quả giá trị đầu ra nhận được là bao nhiêu khi dữ liệu đầu vào hợp lệ?</t>
+          <t>Trong Python 3.x, kết quả trả về của phép chia thực `10 / 2` có kiểu dữ liệu là gì?</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
@@ -597,31 +591,31 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Giá trị được tính toán chính xác theo đúng nhánh rẽ được kích hoạt</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>int (số nguyên)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n"/>
       <c r="B11" s="4" t="n"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Giá trị mặc định ban đầu do biến không được cập nhật</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="n"/>
+          <t>float (số thực)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n"/>
       <c r="B12" s="4" t="n"/>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Báo lỗi Runtime Exception do truy cập biến chưa khởi tạo</t>
+          <t>bool (luận lý)</t>
         </is>
       </c>
       <c r="D12" s="3" t="n"/>
@@ -631,7 +625,7 @@
       <c r="B13" s="4" t="n"/>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Trả về giá trị `None`/`null` do logic rẽ nhánh bị thiếu</t>
+          <t>str (chuỗi)</t>
         </is>
       </c>
       <c r="D13" s="3" t="n"/>
@@ -639,7 +633,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Điểm khác biệt lớn nhất về tính ứng dụng giữa cấu trúc rẽ nhánh cơ bản và cấu trúc lồng nhau trong Toán tử Số học và Toán tử Gán là gì?</t>
+          <t>Toán tử gán gộp `x **= 2` tương đương với câu lệnh nào sau đây?</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
@@ -647,31 +641,31 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Cấu trúc lồng nhau cho phép kiểm tra thêm các điều kiện phụ thuộc khi điều kiện cha thỏa mãn</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>x = x * 2</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n"/>
       <c r="B15" s="4" t="n"/>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Cấu trúc rẽ nhánh cơ bản thực thi nhanh hơn gấp 10 lần cấu trúc lồng nhau</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="n"/>
+          <t>x = x ** 2</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
       <c r="B16" s="4" t="n"/>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Cấu trúc lồng nhau chỉ dùng được cho kiểu dữ liệu chuỗi text</t>
+          <t>x = 2 ** x</t>
         </is>
       </c>
       <c r="D16" s="3" t="n"/>
@@ -681,7 +675,7 @@
       <c r="B17" s="4" t="n"/>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Cấu trúc rẽ nhánh cơ bản không cho phép sử dụng các toán tử so sánh</t>
+          <t>x = x ^ 2</t>
         </is>
       </c>
       <c r="D17" s="3" t="n"/>
@@ -689,7 +683,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Giả sử lập trình viên viết điều kiện trong Toán tử Số học và Toán tử Gán nhưng quên không cập nhật biến đếm hoặc biến điều kiện trong thân khối lệnh. Bẫy lỗi (Pitfall) nào sẽ xảy ra?</t>
+          <t>Khi thực hiện biểu thức `result = 100 / 0` trong Python, chương trình sẽ sinh ra biệt lệ (exception) nào?</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
@@ -697,21 +691,17 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Chương trình rơi vào bẫy lặp vô tận (Infinite Loop) hoặc kết quả bị treo</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>ValueError</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n"/>
       <c r="B19" s="4" t="n"/>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Ngôn ngữ tự động bổ sung câu lệnh cập nhật biến ở background</t>
+          <t>TypeError</t>
         </is>
       </c>
       <c r="D19" s="3" t="n"/>
@@ -721,17 +711,21 @@
       <c r="B20" s="4" t="n"/>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Chương trình tự động bỏ qua khối lệnh và hoàn tất thực thi ngay</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="n"/>
+          <t>ZeroDivisionError</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>
       <c r="B21" s="4" t="n"/>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống sẽ tự động chuyển đổi sang cấu trúc điều khiển khác</t>
+          <t>SyntaxError</t>
         </is>
       </c>
       <c r="D21" s="3" t="n"/>

</xml_diff>